<commit_message>
trial and errror? might reverse....
</commit_message>
<xml_diff>
--- a/prices.xlsx
+++ b/prices.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="105">
   <si>
     <t>Azonosító (ne szerkeszd)</t>
   </si>
@@ -725,7 +725,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F54"/>
+  <dimension ref="A1:F53"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -952,79 +952,76 @@
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="B19" t="s">
-        <v>36</v>
-      </c>
-      <c r="C19" t="s">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="D19" s="4">
-        <v>1200</v>
+        <v>11200</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B20" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D20" s="4">
-        <v>11200</v>
+        <v>2280</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B21" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D21" s="4">
-        <v>2280</v>
+        <v>8850</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B22" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="D22" s="4">
-        <v>8850</v>
+        <v>3500</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B23" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D23" s="4">
-        <v>3500</v>
+        <v>5700</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B24" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="D24" s="4">
-        <v>5700</v>
+        <v>42000</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B25" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D25" s="4">
         <v>42000</v>
@@ -1032,68 +1029,68 @@
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B26" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D26" s="4">
-        <v>42000</v>
+        <v>28000</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B27" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="D27" s="4">
-        <v>28000</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+        <v>21000</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B28" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="D28" s="4">
-        <v>21000</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+        <v>350</v>
+      </c>
+      <c r="E28" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="B29" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="D29" s="4">
-        <v>350</v>
-      </c>
-      <c r="E29" t="s">
-        <v>59</v>
+        <v>3106</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B30" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="D30" s="4">
-        <v>3106</v>
+        <v>3750</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B31" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="D31" s="4">
         <v>3750</v>
@@ -1101,10 +1098,10 @@
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B32" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D32" s="4">
         <v>3750</v>
@@ -1112,142 +1109,142 @@
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B33" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D33" s="4">
-        <v>3750</v>
+        <v>300</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B34" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D34" s="4">
-        <v>300</v>
+        <v>376</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B35" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D35" s="4">
-        <v>376</v>
+        <v>750</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B36" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="D36" s="4">
-        <v>750</v>
+        <v>976</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B37" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="D37" s="4">
-        <v>976</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" s="3" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B38" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="D38" s="4">
-        <v>3000</v>
+        <v>8400</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39" s="3" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B39" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="D39" s="4">
-        <v>8400</v>
+        <v>5250</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" s="3" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B40" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="D40" s="4">
-        <v>5250</v>
+        <v>2500</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" s="3" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B41" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="D41" s="4">
-        <v>2500</v>
+        <v>1050</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42" s="3" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B42" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="D42" s="4">
-        <v>1050</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+        <v>2100</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" s="3" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B43" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D43" s="4">
-        <v>2100</v>
-      </c>
-    </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+        <v>16500</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B44" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D44" s="4">
-        <v>16500</v>
+        <v>17500</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45" s="3" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B45" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="D45" s="4">
         <v>17500</v>
@@ -1255,76 +1252,65 @@
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" s="3" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B46" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D46" s="4">
-        <v>17500</v>
+        <v>28000</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47" s="3" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B47" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="D47" s="4">
-        <v>28000</v>
+        <v>3750</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48" s="3" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B48" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="D48" s="4">
-        <v>3750</v>
+        <v>21000</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" s="3" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B49" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="D49" s="4">
-        <v>21000</v>
-      </c>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+        <v>4800</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" s="3" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B50" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="D50" s="4">
-        <v>4800</v>
-      </c>
-    </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A51" s="3" t="s">
-        <v>102</v>
-      </c>
-      <c r="B51" t="s">
-        <v>103</v>
-      </c>
-      <c r="D51" s="4">
         <v>60000</v>
       </c>
-      <c r="F51" t="s">
+      <c r="F50" t="s">
         <v>104</v>
       </c>
     </row>
+    <row r="51" spans="4:4" x14ac:dyDescent="0.25"/>
     <row r="52" spans="4:4" x14ac:dyDescent="0.25"/>
     <row r="53" spans="4:4" x14ac:dyDescent="0.25"/>
-    <row r="54" spans="4:4" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Most refresh, jo lessze ?
</commit_message>
<xml_diff>
--- a/prices.xlsx
+++ b/prices.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="110">
   <si>
     <t>Azonosító (ne szerkeszd)</t>
   </si>
@@ -145,6 +145,9 @@
     <t>Kerekeskút (GPPB03)</t>
   </si>
   <si>
+    <t>Please request a price!</t>
+  </si>
+  <si>
     <t>garden-daybed</t>
   </si>
   <si>
@@ -197,9 +200,6 @@
   </si>
   <si>
     <t>Tömörfa harangláb (GPSS05)</t>
-  </si>
-  <si>
-    <t>Please request a quote!</t>
   </si>
   <si>
     <t>solid-wood-fence</t>
@@ -744,7 +744,7 @@
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
-    <col min="2" max="2" width="40" customWidth="1"/>
+    <col min="2" max="2" width="43" customWidth="1"/>
     <col min="3" max="3" width="22" customWidth="1"/>
     <col min="4" max="4" width="14" customWidth="1"/>
     <col min="5" max="5" width="10" customWidth="1"/>
@@ -979,23 +979,24 @@
         <v>1200</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
         <v>42</v>
       </c>
       <c r="B20" t="s">
         <v>43</v>
       </c>
-      <c r="D20" s="4">
-        <v>11200</v>
+      <c r="D20" s="4"/>
+      <c r="F20" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B21" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D21" s="4">
         <v>2280</v>
@@ -1003,10 +1004,10 @@
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B22" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D22" s="4">
         <v>8850</v>
@@ -1014,10 +1015,10 @@
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B23" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D23" s="4">
         <v>3500</v>
@@ -1025,10 +1026,10 @@
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B24" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D24" s="4">
         <v>5700</v>
@@ -1036,10 +1037,10 @@
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B25" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D25" s="4">
         <v>42000</v>
@@ -1047,32 +1048,33 @@
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B26" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D26" s="4">
         <v>42000</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B27" t="s">
-        <v>57</v>
-      </c>
-      <c r="D27" s="4">
-        <v>28000</v>
+        <v>58</v>
+      </c>
+      <c r="D27" s="4"/>
+      <c r="F27" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B28" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D28" s="4">
         <v>21000</v>
@@ -1080,16 +1082,13 @@
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B29" t="s">
-        <v>61</v>
-      </c>
-      <c r="D29">
-        <v>60000</v>
+        <v>62</v>
       </c>
       <c r="F29" t="s">
-        <v>62</v>
+        <v>44</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
@@ -1350,6 +1349,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>